<commit_message>
Add SOH report for 2026-10-26
</commit_message>
<xml_diff>
--- a/reports/SOH_26_10_2026.xlsx
+++ b/reports/SOH_26_10_2026.xlsx
@@ -7914,7 +7914,7 @@
         </is>
       </c>
       <c r="D267" s="2" t="n">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E267" s="3" t="n">
         <v>1</v>
@@ -8822,7 +8822,7 @@
         </is>
       </c>
       <c r="D303" s="2" t="n">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="E303" s="3" t="n">
         <v>1</v>
@@ -9410,7 +9410,7 @@
         </is>
       </c>
       <c r="D324" s="2" t="n">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E324" s="3" t="n">
         <v>1</v>
@@ -10782,7 +10782,7 @@
         </is>
       </c>
       <c r="D373" s="2" t="n">
-        <v>1455</v>
+        <v>1454</v>
       </c>
       <c r="E373" s="3" t="n">
         <v>40000</v>
@@ -10838,7 +10838,7 @@
         </is>
       </c>
       <c r="D375" s="2" t="n">
-        <v>1082</v>
+        <v>1080</v>
       </c>
       <c r="E375" s="3" t="n">
         <v>40000</v>
@@ -11454,7 +11454,7 @@
         </is>
       </c>
       <c r="D397" s="2" t="n">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="E397" s="3" t="n">
         <v>51000</v>
@@ -18874,7 +18874,7 @@
         </is>
       </c>
       <c r="D662" s="2" t="n">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="E662" s="3" t="n">
         <v>1</v>
@@ -25650,7 +25650,7 @@
         </is>
       </c>
       <c r="D904" s="2" t="n">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="E904" s="3" t="n">
         <v>1</v>
@@ -25958,7 +25958,7 @@
         </is>
       </c>
       <c r="D915" s="2" t="n">
-        <v>899</v>
+        <v>898</v>
       </c>
       <c r="E915" s="3" t="n">
         <v>12500</v>

</xml_diff>